<commit_message>
docs: add AG topology to solver-integration spec and sample (per-machine AG + HW_Caps)
Fault domain = AG; HW_Current gains a trailing ag column (forward-compatible: current importer reads first 4 cols, ignores ag), new HW_Caps sheet for per-AG slot caps. Fabs hosting control-plane new-builds get >=5 AGs (master x5 spread). Spec updated with topology mapping (procurement_spread_dimension=ag).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/v2_sample_solver.xlsx
+++ b/examples/v2_sample_solver.xlsx
@@ -13,8 +13,9 @@
     <sheet name="HW_SKU" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="HW_Current" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="HW_MoveIn" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cluster_Menu" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="New_Build" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="HW_Caps" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cluster_Menu" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="New_Build" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -809,7 +810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -833,6 +834,11 @@
           <t>count</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ag</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -851,7 +857,12 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ag1</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -867,17 +878,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>big-128</t>
+          <t>std-64</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ag2</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -891,27 +907,237 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>2</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ag3</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>big-128</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ag1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>big-128</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ag2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>big-128</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ag3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>std-64</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ag1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>std-64</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ag2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>std-64</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ag3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>network2</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>std-64</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>5</v>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ag1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>std-64</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ag2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>std-64</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ag3</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -991,33 +1217,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>menu</t>
+          <t>fab</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>network</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>ag</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>co_residency</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>vm_vcore</t>
+          <t>max_bm</t>
         </is>
       </c>
     </row>
@@ -1029,19 +1250,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>master</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>16</v>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ag1</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -1052,19 +1270,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>infra</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>8</v>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ag2</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -1075,19 +1290,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>l4lb</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>8</v>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ag3</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -1098,42 +1310,36 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>learner</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>5</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>32</v>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ag4</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>master</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>16</v>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ag5</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="7">
@@ -1144,19 +1350,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>infra</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>8</v>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ag1</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -1167,19 +1370,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>l4lb</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>8</v>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ag2</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -1190,42 +1390,36 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>learner</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>5</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>32</v>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ag3</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>exclusive</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>32</v>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ag1</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -1236,19 +1430,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>master</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>5</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>16</v>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ag2</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="12">
@@ -1259,19 +1450,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>infra</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>8</v>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ag3</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="13">
@@ -1282,19 +1470,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>l4lb</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>8</v>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ag4</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="14">
@@ -1305,364 +1490,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>learner</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Bastion</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>exclusive</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>master</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>5</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>infra</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>5</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>l4lb</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>3</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>learner</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>5</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>3</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>exclusive</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Bastion</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>exclusive</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>master</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>5</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>infra</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>5</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>l4lb</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>3</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>learner</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>5</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>shared</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>3</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>exclusive</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Bastion</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>exclusive</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>3</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>exclusive</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>VT</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>3</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>exclusive</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>16</v>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ag5</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1676,6 +1513,691 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>menu</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>co_residency</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>vm_vcore</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>master</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>infra</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>l4lb</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>learner</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>master</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>infra</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>l4lb</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>learner</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>exclusive</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>master</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>infra</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>l4lb</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>learner</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Bastion</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>exclusive</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>master</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>infra</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>5</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>l4lb</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>learner</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>exclusive</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bastion</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>exclusive</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>master</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>5</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>infra</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>l4lb</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>learner</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>exclusive</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Bastion</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>exclusive</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HA</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>exclusive</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>exclusive</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
feat: unified fab-tab layout (Menu column) + rich scenario sample; adapter maps detail worker
models: MoveIn.ag, NewBuild, PlanInput.new_builds/menus. importer: Menu column (F) in fab tabs classifies Worker vs new-build (months shift to G), captures new_builds, parses Cluster_Menu into menus dict, reads optional HW_MoveIn ag. generator: unified layout with varied scenarios in A/B/C (coarse/detail worker, blast radius, free/exclusive/group tenant, new-build menus A/B/D/E, single/multi-cluster build months). adapter: also maps detail worker vm_demands (fixed count x size) to demand_book. Live-verified (7 fab-periods feasible incl. detail worker). Blast-radius/tenant enforcement + control-plane expansion still pending §6.2.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/v2_sample_solver.xlsx
+++ b/examples/v2_sample_solver.xlsx
@@ -15,7 +15,6 @@
     <sheet name="HW_MoveIn" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="HW_Caps" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Cluster_Menu" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="New_Build" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37,12 +36,18 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+        <bgColor rgb="00DDEBF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -57,9 +62,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:Y5"/>
+  <dimension ref="A4:Y10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -446,25 +452,30 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>每台上限</t>
+          <t>爆炸半徑 (1:x), EX: 2</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>共居</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
+          <t>Tenant (自由=留空/指定群組/獨佔)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
@@ -503,7 +514,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>web-svc</t>
+          <t>web</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -511,11 +522,171 @@
           <t>network1</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Worker</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
         <v>200</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>120</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>old-a</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>std-64</t>
+        </is>
+      </c>
+      <c r="W5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>cache</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>60</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Worker</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>180</v>
+      </c>
+      <c r="H6" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>iso</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>51</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>獨佔</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Worker</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>48</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>teamA</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Worker</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>144</v>
+      </c>
+      <c r="H8" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>c-happy</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>c-lite</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -529,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:Y5"/>
+  <dimension ref="A4:Y6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -550,25 +721,30 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>每台上限</t>
+          <t>爆炸半徑 (1:x), EX: 2</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>共居</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
+          <t>Tenant (自由=留空/指定群組/獨佔)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
@@ -615,14 +791,60 @@
           <t>network1</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>300</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Worker</t>
+        </is>
       </c>
       <c r="G5" t="n">
         <v>300</v>
       </c>
       <c r="H5" t="n">
         <v>300</v>
+      </c>
+      <c r="I5" t="n">
+        <v>300</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>old-b</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>std-64</t>
+        </is>
+      </c>
+      <c r="Y5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>c-mega</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -636,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:Y5"/>
+  <dimension ref="A4:Y6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -657,25 +879,30 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>每台上限</t>
+          <t>爆炸半徑 (1:x), EX: 2</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>共居</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
+          <t>Tenant (自由=留空/指定群組/獨佔)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
@@ -722,11 +949,45 @@
           <t>network2</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="C5" t="n">
+        <v>32</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Worker</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
         <v>150</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>150</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>c-twin</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -810,7 +1071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -973,32 +1234,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>network1</t>
+          <t>network2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>big-128</t>
+          <t>std-64</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ag3</t>
+          <t>ag1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>network1</t>
+          <t>network2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1007,11 +1268,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ag1</t>
+          <t>ag2</t>
         </is>
       </c>
     </row>
@@ -1032,11 +1293,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ag2</t>
+          <t>ag1</t>
         </is>
       </c>
     </row>
@@ -1061,19 +1322,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ag3</t>
+          <t>ag2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>network2</t>
+          <t>network1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1082,11 +1343,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ag1</t>
+          <t>ag3</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1372,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ag2</t>
+          <t>ag1</t>
         </is>
       </c>
     </row>
@@ -1132,9 +1393,34 @@
         </is>
       </c>
       <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ag2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>std-64</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
         <v>1</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>ag3</t>
         </is>
@@ -1151,7 +1437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1180,6 +1466,11 @@
           <t>count</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ag</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1204,6 +1495,11 @@
       </c>
       <c r="E2" t="n">
         <v>2</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ag1</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1217,7 +1513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1345,12 +1641,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>network1</t>
+          <t>network2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1365,12 +1661,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>network1</t>
+          <t>network2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1385,12 +1681,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>network1</t>
+          <t>network2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1405,7 +1701,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1415,7 +1711,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ag1</t>
+          <t>ag4</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1425,7 +1721,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1435,7 +1731,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ag2</t>
+          <t>ag5</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1445,17 +1741,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>network2</t>
+          <t>network1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ag3</t>
+          <t>ag1</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1465,17 +1761,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>network2</t>
+          <t>network1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ag4</t>
+          <t>ag2</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1485,20 +1781,120 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>network1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ag3</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>network2</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ag1</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ag2</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ag3</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ag4</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>network2</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>ag5</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D19" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2190,99 +2586,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>fab</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>network</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>cluster</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>menu</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>network1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>c2</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>network2</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>c5</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: regenerate v2 sample with return-AG column
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/v2_sample_solver.xlsx
+++ b/examples/v2_sample_solver.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:Y10"/>
+  <dimension ref="A4:Z10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -495,17 +495,22 @@
           <t>機型</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="W4" s="1" t="inlineStr">
+        <is>
+          <t>ag</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
@@ -548,7 +553,12 @@
           <t>std-64</t>
         </is>
       </c>
-      <c r="W5" t="n">
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>ag1</t>
+        </is>
+      </c>
+      <c r="X5" t="n">
         <v>3</v>
       </c>
     </row>
@@ -700,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:Y6"/>
+  <dimension ref="A4:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -764,17 +774,22 @@
           <t>機型</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="W4" s="1" t="inlineStr">
+        <is>
+          <t>ag</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
@@ -820,7 +835,12 @@
           <t>std-64</t>
         </is>
       </c>
-      <c r="Y5" t="n">
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>ag2</t>
+        </is>
+      </c>
+      <c r="Z5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -858,7 +878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:Y6"/>
+  <dimension ref="A4:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -922,17 +942,22 @@
           <t>機型</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="W4" s="1" t="inlineStr">
+        <is>
+          <t>ag</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>

</xml_diff>